<commit_message>
Atualização de dados - Ref. Junho/26
</commit_message>
<xml_diff>
--- a/data/Custos OMIE.xlsx
+++ b/data/Custos OMIE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Brsrvfs\arquivos\PROJETOS\Dashboards\Painel Gerencial\OMIE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFFF640-F63B-48BB-94FD-D50072F7AED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA61D358-6BFA-48DB-9C8C-61859583F5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="4" xr2:uid="{4CA471FC-88D0-4035-A554-576A2C9AB245}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{4CA471FC-88D0-4035-A554-576A2C9AB245}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos jan26" sheetId="1" r:id="rId1"/>
@@ -18,11 +18,13 @@
     <sheet name="Custos mar26" sheetId="3" r:id="rId3"/>
     <sheet name="Custos abr26" sheetId="4" r:id="rId4"/>
     <sheet name="Custos mai26" sheetId="5" r:id="rId5"/>
+    <sheet name="Custos jun26" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="data" localSheetId="3">'Custos abr26'!$A$1:$C$15</definedName>
     <definedName name="data" localSheetId="1">'Custos fev26'!$A$1:$C$15</definedName>
     <definedName name="data" localSheetId="0">'Custos jan26'!#REF!</definedName>
+    <definedName name="data" localSheetId="5">'Custos jun26'!$A$1:$C$15</definedName>
     <definedName name="data" localSheetId="4">'Custos mai26'!$A$1:$C$15</definedName>
     <definedName name="data" localSheetId="2">'Custos mar26'!$A$1:$C$15</definedName>
     <definedName name="data_1" localSheetId="0">'Custos jan26'!$A$1:$C$15</definedName>
@@ -83,11 +85,20 @@
       </textFields>
     </textPr>
   </connection>
+  <connection id="6" xr16:uid="{B3797530-14AC-4EC4-89CF-1BB4A1B0586B}" name="data6" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr codePage="65001" sourceFile="C:\Users\Bruno Dalmeida\Downloads\data.csv" decimal="," thousands="." tab="0" comma="1">
+      <textFields count="3">
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
 </connections>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="17">
   <si>
     <t>Grupo Resumo Final</t>
   </si>
@@ -211,6 +222,10 @@
 
 <file path=xl/queryTables/queryTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="data" connectionId="5" xr16:uid="{BBCC69F4-423E-4553-ABAC-4A6512542568}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="data" connectionId="6" xr16:uid="{F11BB640-DDC4-4EC1-8B4E-6A0ADC20B426}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1406,4 +1421,184 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EAE60C-B2BD-4AF5-9AA6-FF644DDD6E4B}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>1829412.28</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.38869999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>865240.78</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.18379999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>690945.93</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.14680000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>426175.74</v>
+      </c>
+      <c r="C5" s="1">
+        <v>9.06E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>333277.82</v>
+      </c>
+      <c r="C6" s="1">
+        <v>7.0800000000000002E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>232498.9</v>
+      </c>
+      <c r="C7" s="1">
+        <v>4.9399999999999999E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>79908.23</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.7000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>67402.59</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.43E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>64549.05</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1.37E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>43975.35</v>
+      </c>
+      <c r="C11" s="1">
+        <v>9.2999999999999992E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>42729.120000000003</v>
+      </c>
+      <c r="C12" s="1">
+        <v>9.1000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>11238.82</v>
+      </c>
+      <c r="C13" s="1">
+        <v>2.3999999999999998E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>10531.35</v>
+      </c>
+      <c r="C14" s="1">
+        <v>2.2000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>8513.98</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1.8E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>